<commit_message>
abhi to shuru huwa h
</commit_message>
<xml_diff>
--- a/runs/registry/attendance.xlsx
+++ b/runs/registry/attendance.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -825,6 +825,60 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Aayush</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2025-09-07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>22:14:50</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>voice+face agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Aayush</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>09:42:14</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>voice+face agree</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
integrating the agentic AI
</commit_message>
<xml_diff>
--- a/runs/registry/attendance.xlsx
+++ b/runs/registry/attendance.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -879,6 +879,114 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Aayush</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>12:22:15</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>voice+face agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Aayush</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>12:22:23</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>voice+face agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Aayush</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>12:22:31</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>voice+face agree</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Aayush</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2025-09-08</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>12:22:40</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>voice+face agree</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>